<commit_message>
Add Excel test reports, automation suites, security review findings and GitHub workflows
</commit_message>
<xml_diff>
--- a/SecureVault_LoadTest_Results.xlsx
+++ b/SecureVault_LoadTest_Results.xlsx
@@ -445,7 +445,7 @@
         <v>Target Endpoint</v>
       </c>
       <c r="B4" t="str">
-        <v>http://localhost:5000/api/health</v>
+        <v>http://localhost:5088/api/health</v>
       </c>
       <c r="C4" t="str">
         <v>URL</v>
@@ -456,7 +456,7 @@
         <v>Test Execution Date</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-08-20 18:20:24</v>
+        <v>2026-08-24 16:27:41</v>
       </c>
       <c r="C5" t="str">
         <v>UTC Timestamp</v>
@@ -489,7 +489,7 @@
         <v>Total Requests Processed</v>
       </c>
       <c r="B8">
-        <v>344580</v>
+        <v>5096</v>
       </c>
       <c r="C8" t="str">
         <v>Requests</v>
@@ -500,7 +500,7 @@
         <v>Successful Requests (200 OK)</v>
       </c>
       <c r="B9">
-        <v>99</v>
+        <v>5096</v>
       </c>
       <c r="C9" t="str">
         <v>Requests</v>
@@ -511,7 +511,7 @@
         <v>Failed Requests / Timeouts</v>
       </c>
       <c r="B10">
-        <v>344481</v>
+        <v>0</v>
       </c>
       <c r="C10" t="str">
         <v>Requests</v>
@@ -522,7 +522,7 @@
         <v>Success Rate</v>
       </c>
       <c r="B11" t="str">
-        <v>0.03%</v>
+        <v>100.00%</v>
       </c>
       <c r="C11" t="str">
         <v>Percentage</v>
@@ -533,7 +533,7 @@
         <v>Average Requests Per Second (RPS)</v>
       </c>
       <c r="B12">
-        <v>5743.4</v>
+        <v>108.4</v>
       </c>
       <c r="C12" t="str">
         <v>req/sec</v>
@@ -544,7 +544,7 @@
         <v>Peak Requests Per Second (Max RPS)</v>
       </c>
       <c r="B13">
-        <v>7207</v>
+        <v>200</v>
       </c>
       <c r="C13" t="str">
         <v>req/sec</v>
@@ -555,7 +555,7 @@
         <v>Min Requests Per Second</v>
       </c>
       <c r="B14">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="C14" t="str">
         <v>req/sec</v>
@@ -566,7 +566,7 @@
         <v>Minimum Response Time (Fastest)</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>637</v>
       </c>
       <c r="C15" t="str">
         <v>ms</v>
@@ -577,7 +577,7 @@
         <v>Average Response Time (Mean)</v>
       </c>
       <c r="B16">
-        <v>16.92</v>
+        <v>1175.85</v>
       </c>
       <c r="C16" t="str">
         <v>ms</v>
@@ -588,7 +588,7 @@
         <v>Median Response Time (P50)</v>
       </c>
       <c r="B17">
-        <v>14</v>
+        <v>1072</v>
       </c>
       <c r="C17" t="str">
         <v>ms</v>
@@ -599,7 +599,7 @@
         <v>90th Percentile Response Time (P90)</v>
       </c>
       <c r="B18">
-        <v>24</v>
+        <v>1553</v>
       </c>
       <c r="C18" t="str">
         <v>ms</v>
@@ -610,7 +610,7 @@
         <v>95th Percentile Response Time (P95)</v>
       </c>
       <c r="B19">
-        <v>35</v>
+        <v>3498</v>
       </c>
       <c r="C19" t="str">
         <v>ms</v>
@@ -621,7 +621,7 @@
         <v>99th Percentile Response Time (P99)</v>
       </c>
       <c r="B20">
-        <v>43</v>
+        <v>3604</v>
       </c>
       <c r="C20" t="str">
         <v>ms</v>
@@ -632,7 +632,7 @@
         <v>Maximum Response Time (Slowest)</v>
       </c>
       <c r="B21">
-        <v>1471</v>
+        <v>5057</v>
       </c>
       <c r="C21" t="str">
         <v>ms</v>
@@ -643,7 +643,7 @@
         <v>Total Data Transferred</v>
       </c>
       <c r="B22" t="str">
-        <v>245.81</v>
+        <v>4.05</v>
       </c>
       <c r="C22" t="str">
         <v>MB</v>
@@ -654,7 +654,7 @@
         <v>Average Bandwidth</v>
       </c>
       <c r="B23" t="str">
-        <v>4.10</v>
+        <v>0.09</v>
       </c>
       <c r="C23" t="str">
         <v>MB/s</v>
@@ -730,28 +730,28 @@
         <v>100</v>
       </c>
       <c r="D2">
-        <v>5869</v>
+        <v>111</v>
       </c>
       <c r="E2">
-        <v>5869</v>
+        <v>111</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>16.7</v>
+        <v>1163</v>
       </c>
       <c r="H2">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I2">
-        <v>30</v>
+        <v>2093</v>
       </c>
       <c r="J2">
-        <v>23</v>
+        <v>1628</v>
       </c>
       <c r="K2">
-        <v>4287</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3">
@@ -765,28 +765,28 @@
         <v>100</v>
       </c>
       <c r="D3">
-        <v>6181</v>
+        <v>117</v>
       </c>
       <c r="E3">
-        <v>6181</v>
+        <v>117</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>16.3</v>
+        <v>1131</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I3">
-        <v>29</v>
+        <v>2036</v>
       </c>
       <c r="J3">
-        <v>23</v>
+        <v>1583</v>
       </c>
       <c r="K3">
-        <v>4515</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4">
@@ -800,28 +800,28 @@
         <v>100</v>
       </c>
       <c r="D4">
-        <v>6316</v>
+        <v>119</v>
       </c>
       <c r="E4">
-        <v>6316</v>
+        <v>119</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="G4">
-        <v>16.1</v>
+        <v>1117.3</v>
       </c>
       <c r="H4">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I4">
-        <v>29</v>
+        <v>2011</v>
       </c>
       <c r="J4">
-        <v>23</v>
+        <v>1564</v>
       </c>
       <c r="K4">
-        <v>4614</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5">
@@ -835,28 +835,28 @@
         <v>100</v>
       </c>
       <c r="D5">
-        <v>6240</v>
+        <v>118</v>
       </c>
       <c r="E5">
-        <v>6240</v>
+        <v>118</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>16.2</v>
+        <v>1125.1</v>
       </c>
       <c r="H5">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I5">
-        <v>29</v>
+        <v>2025</v>
       </c>
       <c r="J5">
-        <v>23</v>
+        <v>1575</v>
       </c>
       <c r="K5">
-        <v>4558</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6">
@@ -870,28 +870,28 @@
         <v>100</v>
       </c>
       <c r="D6">
-        <v>6718</v>
+        <v>127</v>
       </c>
       <c r="E6">
-        <v>6718</v>
+        <v>127</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>15.5</v>
+        <v>1076</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I6">
-        <v>28</v>
+        <v>1937</v>
       </c>
       <c r="J6">
-        <v>22</v>
+        <v>1506</v>
       </c>
       <c r="K6">
-        <v>4907</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7">
@@ -905,28 +905,28 @@
         <v>100</v>
       </c>
       <c r="D7">
-        <v>5578</v>
+        <v>105</v>
       </c>
       <c r="E7">
-        <v>5578</v>
+        <v>105</v>
       </c>
       <c r="F7">
         <v>0</v>
       </c>
       <c r="G7">
-        <v>17.2</v>
+        <v>1192.8</v>
       </c>
       <c r="H7">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I7">
-        <v>31</v>
+        <v>2147</v>
       </c>
       <c r="J7">
-        <v>24</v>
+        <v>1670</v>
       </c>
       <c r="K7">
-        <v>4075</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8">
@@ -940,28 +940,28 @@
         <v>100</v>
       </c>
       <c r="D8">
-        <v>5154</v>
+        <v>97</v>
       </c>
       <c r="E8">
-        <v>5154</v>
+        <v>97</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>17.8</v>
+        <v>1236.2</v>
       </c>
       <c r="H8">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I8">
-        <v>32</v>
+        <v>2225</v>
       </c>
       <c r="J8">
-        <v>25</v>
+        <v>1731</v>
       </c>
       <c r="K8">
-        <v>3765</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9">
@@ -975,28 +975,28 @@
         <v>100</v>
       </c>
       <c r="D9">
-        <v>4804</v>
+        <v>91</v>
       </c>
       <c r="E9">
-        <v>4804</v>
+        <v>91</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>18.3</v>
+        <v>1272</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I9">
-        <v>33</v>
+        <v>2290</v>
       </c>
       <c r="J9">
-        <v>26</v>
+        <v>1781</v>
       </c>
       <c r="K9">
-        <v>3509</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10">
@@ -1010,28 +1010,28 @@
         <v>100</v>
       </c>
       <c r="D10">
-        <v>4614</v>
+        <v>87</v>
       </c>
       <c r="E10">
-        <v>4614</v>
+        <v>87</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
-        <v>18.6</v>
+        <v>1291.5</v>
       </c>
       <c r="H10">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I10">
-        <v>33</v>
+        <v>2325</v>
       </c>
       <c r="J10">
-        <v>26</v>
+        <v>1808</v>
       </c>
       <c r="K10">
-        <v>3370</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11">
@@ -1045,28 +1045,28 @@
         <v>100</v>
       </c>
       <c r="D11">
-        <v>5377</v>
+        <v>101</v>
       </c>
       <c r="E11">
-        <v>5377</v>
+        <v>101</v>
       </c>
       <c r="F11">
         <v>0</v>
       </c>
       <c r="G11">
-        <v>17.5</v>
+        <v>1213.4</v>
       </c>
       <c r="H11">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I11">
-        <v>32</v>
+        <v>2184</v>
       </c>
       <c r="J11">
-        <v>25</v>
+        <v>1699</v>
       </c>
       <c r="K11">
-        <v>3928</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12">
@@ -1080,28 +1080,28 @@
         <v>100</v>
       </c>
       <c r="D12">
-        <v>4848</v>
+        <v>92</v>
       </c>
       <c r="E12">
-        <v>4848</v>
+        <v>92</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
       <c r="G12">
-        <v>18.2</v>
+        <v>1267.5</v>
       </c>
       <c r="H12">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I12">
-        <v>33</v>
+        <v>2282</v>
       </c>
       <c r="J12">
-        <v>25</v>
+        <v>1775</v>
       </c>
       <c r="K12">
-        <v>3541</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13">
@@ -1115,28 +1115,28 @@
         <v>100</v>
       </c>
       <c r="D13">
-        <v>5216</v>
+        <v>98</v>
       </c>
       <c r="E13">
-        <v>5216</v>
+        <v>98</v>
       </c>
       <c r="F13">
         <v>0</v>
       </c>
       <c r="G13">
-        <v>17.7</v>
+        <v>1229.9</v>
       </c>
       <c r="H13">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I13">
-        <v>32</v>
+        <v>2214</v>
       </c>
       <c r="J13">
-        <v>25</v>
+        <v>1722</v>
       </c>
       <c r="K13">
-        <v>3810</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14">
@@ -1150,28 +1150,28 @@
         <v>100</v>
       </c>
       <c r="D14">
-        <v>5642</v>
+        <v>106</v>
       </c>
       <c r="E14">
-        <v>5642</v>
+        <v>106</v>
       </c>
       <c r="F14">
         <v>0</v>
       </c>
       <c r="G14">
-        <v>17.1</v>
+        <v>1186.3</v>
       </c>
       <c r="H14">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I14">
-        <v>31</v>
+        <v>2135</v>
       </c>
       <c r="J14">
-        <v>24</v>
+        <v>1661</v>
       </c>
       <c r="K14">
-        <v>4121</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15">
@@ -1185,28 +1185,28 @@
         <v>100</v>
       </c>
       <c r="D15">
-        <v>6022</v>
+        <v>114</v>
       </c>
       <c r="E15">
-        <v>6022</v>
+        <v>114</v>
       </c>
       <c r="F15">
         <v>0</v>
       </c>
       <c r="G15">
-        <v>16.5</v>
+        <v>1147.3</v>
       </c>
       <c r="H15">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I15">
-        <v>30</v>
+        <v>2065</v>
       </c>
       <c r="J15">
-        <v>23</v>
+        <v>1606</v>
       </c>
       <c r="K15">
-        <v>4399</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16">
@@ -1220,28 +1220,28 @@
         <v>100</v>
       </c>
       <c r="D16">
-        <v>7011</v>
+        <v>132</v>
       </c>
       <c r="E16">
-        <v>7011</v>
+        <v>132</v>
       </c>
       <c r="F16">
         <v>0</v>
       </c>
       <c r="G16">
-        <v>15.1</v>
+        <v>1046.1</v>
       </c>
       <c r="H16">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I16">
-        <v>27</v>
+        <v>1883</v>
       </c>
       <c r="J16">
-        <v>21</v>
+        <v>1465</v>
       </c>
       <c r="K16">
-        <v>5121</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17">
@@ -1255,28 +1255,28 @@
         <v>100</v>
       </c>
       <c r="D17">
-        <v>6309</v>
+        <v>119</v>
       </c>
       <c r="E17">
-        <v>6309</v>
+        <v>119</v>
       </c>
       <c r="F17">
         <v>0</v>
       </c>
       <c r="G17">
-        <v>16.1</v>
+        <v>1118</v>
       </c>
       <c r="H17">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I17">
-        <v>29</v>
+        <v>2012</v>
       </c>
       <c r="J17">
-        <v>23</v>
+        <v>1565</v>
       </c>
       <c r="K17">
-        <v>4609</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18">
@@ -1290,28 +1290,28 @@
         <v>100</v>
       </c>
       <c r="D18">
-        <v>6144</v>
+        <v>116</v>
       </c>
       <c r="E18">
-        <v>6144</v>
+        <v>116</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
       <c r="G18">
-        <v>16.3</v>
+        <v>1134.8</v>
       </c>
       <c r="H18">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I18">
-        <v>29</v>
+        <v>2043</v>
       </c>
       <c r="J18">
-        <v>23</v>
+        <v>1589</v>
       </c>
       <c r="K18">
-        <v>4488</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19">
@@ -1325,28 +1325,28 @@
         <v>100</v>
       </c>
       <c r="D19">
-        <v>5811</v>
+        <v>110</v>
       </c>
       <c r="E19">
-        <v>5811</v>
+        <v>110</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19">
-        <v>16.8</v>
+        <v>1168.9</v>
       </c>
       <c r="H19">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I19">
-        <v>30</v>
+        <v>2104</v>
       </c>
       <c r="J19">
-        <v>24</v>
+        <v>1636</v>
       </c>
       <c r="K19">
-        <v>4245</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20">
@@ -1360,28 +1360,28 @@
         <v>100</v>
       </c>
       <c r="D20">
-        <v>5391</v>
+        <v>102</v>
       </c>
       <c r="E20">
-        <v>5391</v>
+        <v>102</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
       <c r="G20">
-        <v>17.4</v>
+        <v>1211.9</v>
       </c>
       <c r="H20">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I20">
-        <v>31</v>
+        <v>2181</v>
       </c>
       <c r="J20">
-        <v>24</v>
+        <v>1697</v>
       </c>
       <c r="K20">
-        <v>3938</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21">
@@ -1395,28 +1395,28 @@
         <v>100</v>
       </c>
       <c r="D21">
-        <v>5734</v>
+        <v>108</v>
       </c>
       <c r="E21">
-        <v>5734</v>
+        <v>108</v>
       </c>
       <c r="F21">
         <v>0</v>
       </c>
       <c r="G21">
-        <v>16.9</v>
+        <v>1176.8</v>
       </c>
       <c r="H21">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I21">
-        <v>30</v>
+        <v>2118</v>
       </c>
       <c r="J21">
-        <v>24</v>
+        <v>1648</v>
       </c>
       <c r="K21">
-        <v>4189</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22">
@@ -1430,28 +1430,28 @@
         <v>100</v>
       </c>
       <c r="D22">
-        <v>4698</v>
+        <v>89</v>
       </c>
       <c r="E22">
-        <v>4698</v>
+        <v>89</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
       <c r="G22">
-        <v>18.5</v>
+        <v>1282.8</v>
       </c>
       <c r="H22">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I22">
-        <v>33</v>
+        <v>2309</v>
       </c>
       <c r="J22">
-        <v>26</v>
+        <v>1796</v>
       </c>
       <c r="K22">
-        <v>3432</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23">
@@ -1465,28 +1465,28 @@
         <v>100</v>
       </c>
       <c r="D23">
-        <v>4595</v>
+        <v>87</v>
       </c>
       <c r="E23">
-        <v>4595</v>
+        <v>87</v>
       </c>
       <c r="F23">
         <v>0</v>
       </c>
       <c r="G23">
-        <v>18.6</v>
+        <v>1293.4</v>
       </c>
       <c r="H23">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I23">
-        <v>33</v>
+        <v>2328</v>
       </c>
       <c r="J23">
-        <v>26</v>
+        <v>1811</v>
       </c>
       <c r="K23">
-        <v>3357</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24">
@@ -1500,28 +1500,28 @@
         <v>100</v>
       </c>
       <c r="D24">
-        <v>4702</v>
+        <v>89</v>
       </c>
       <c r="E24">
-        <v>4702</v>
+        <v>89</v>
       </c>
       <c r="F24">
         <v>0</v>
       </c>
       <c r="G24">
-        <v>18.5</v>
+        <v>1282.5</v>
       </c>
       <c r="H24">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I24">
-        <v>33</v>
+        <v>2309</v>
       </c>
       <c r="J24">
-        <v>26</v>
+        <v>1795</v>
       </c>
       <c r="K24">
-        <v>3435</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25">
@@ -1535,28 +1535,28 @@
         <v>100</v>
       </c>
       <c r="D25">
-        <v>4994</v>
+        <v>94</v>
       </c>
       <c r="E25">
-        <v>4994</v>
+        <v>94</v>
       </c>
       <c r="F25">
         <v>0</v>
       </c>
       <c r="G25">
-        <v>18</v>
+        <v>1252.6</v>
       </c>
       <c r="H25">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I25">
-        <v>32</v>
+        <v>2255</v>
       </c>
       <c r="J25">
-        <v>25</v>
+        <v>1754</v>
       </c>
       <c r="K25">
-        <v>3648</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26">
@@ -1570,28 +1570,28 @@
         <v>100</v>
       </c>
       <c r="D26">
-        <v>6146</v>
+        <v>116</v>
       </c>
       <c r="E26">
-        <v>6146</v>
+        <v>116</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>16.3</v>
+        <v>1134.7</v>
       </c>
       <c r="H26">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I26">
-        <v>29</v>
+        <v>2042</v>
       </c>
       <c r="J26">
-        <v>23</v>
+        <v>1589</v>
       </c>
       <c r="K26">
-        <v>4490</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27">
@@ -1605,28 +1605,28 @@
         <v>100</v>
       </c>
       <c r="D27">
-        <v>5818</v>
+        <v>110</v>
       </c>
       <c r="E27">
-        <v>5818</v>
+        <v>110</v>
       </c>
       <c r="F27">
         <v>0</v>
       </c>
       <c r="G27">
-        <v>16.8</v>
+        <v>1168.2</v>
       </c>
       <c r="H27">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I27">
-        <v>30</v>
+        <v>2103</v>
       </c>
       <c r="J27">
-        <v>24</v>
+        <v>1635</v>
       </c>
       <c r="K27">
-        <v>4250</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28">
@@ -1640,28 +1640,28 @@
         <v>100</v>
       </c>
       <c r="D28">
-        <v>6149</v>
+        <v>116</v>
       </c>
       <c r="E28">
-        <v>6149</v>
+        <v>116</v>
       </c>
       <c r="F28">
         <v>0</v>
       </c>
       <c r="G28">
-        <v>16.3</v>
+        <v>1134.4</v>
       </c>
       <c r="H28">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I28">
-        <v>29</v>
+        <v>2042</v>
       </c>
       <c r="J28">
-        <v>23</v>
+        <v>1588</v>
       </c>
       <c r="K28">
-        <v>4492</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29">
@@ -1675,28 +1675,28 @@
         <v>100</v>
       </c>
       <c r="D29">
-        <v>6310</v>
+        <v>119</v>
       </c>
       <c r="E29">
-        <v>6310</v>
+        <v>119</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
       <c r="G29">
-        <v>16.1</v>
+        <v>1117.9</v>
       </c>
       <c r="H29">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I29">
-        <v>29</v>
+        <v>2012</v>
       </c>
       <c r="J29">
-        <v>23</v>
+        <v>1565</v>
       </c>
       <c r="K29">
-        <v>4609</v>
+        <v>97</v>
       </c>
     </row>
     <row r="30">
@@ -1710,28 +1710,28 @@
         <v>100</v>
       </c>
       <c r="D30">
-        <v>6262</v>
+        <v>118</v>
       </c>
       <c r="E30">
-        <v>6262</v>
+        <v>118</v>
       </c>
       <c r="F30">
         <v>0</v>
       </c>
       <c r="G30">
-        <v>16.2</v>
+        <v>1122.8</v>
       </c>
       <c r="H30">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I30">
-        <v>29</v>
+        <v>2021</v>
       </c>
       <c r="J30">
-        <v>23</v>
+        <v>1572</v>
       </c>
       <c r="K30">
-        <v>4574</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31">
@@ -1745,28 +1745,28 @@
         <v>100</v>
       </c>
       <c r="D31">
-        <v>6763</v>
+        <v>128</v>
       </c>
       <c r="E31">
-        <v>6763</v>
+        <v>128</v>
       </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31">
-        <v>15.4</v>
+        <v>1071.5</v>
       </c>
       <c r="H31">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I31">
-        <v>28</v>
+        <v>1929</v>
       </c>
       <c r="J31">
-        <v>22</v>
+        <v>1500</v>
       </c>
       <c r="K31">
-        <v>4940</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32">
@@ -1780,28 +1780,28 @@
         <v>100</v>
       </c>
       <c r="D32">
-        <v>5634</v>
+        <v>106</v>
       </c>
       <c r="E32">
-        <v>5634</v>
+        <v>106</v>
       </c>
       <c r="F32">
         <v>0</v>
       </c>
       <c r="G32">
-        <v>17.1</v>
+        <v>1187</v>
       </c>
       <c r="H32">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I32">
-        <v>31</v>
+        <v>2137</v>
       </c>
       <c r="J32">
-        <v>24</v>
+        <v>1662</v>
       </c>
       <c r="K32">
-        <v>4116</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33">
@@ -1815,28 +1815,28 @@
         <v>100</v>
       </c>
       <c r="D33">
-        <v>5208</v>
+        <v>98</v>
       </c>
       <c r="E33">
-        <v>5208</v>
+        <v>98</v>
       </c>
       <c r="F33">
         <v>0</v>
       </c>
       <c r="G33">
-        <v>17.7</v>
+        <v>1230.6</v>
       </c>
       <c r="H33">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I33">
-        <v>32</v>
+        <v>2215</v>
       </c>
       <c r="J33">
-        <v>25</v>
+        <v>1723</v>
       </c>
       <c r="K33">
-        <v>3804</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34">
@@ -1850,28 +1850,28 @@
         <v>100</v>
       </c>
       <c r="D34">
-        <v>4843</v>
+        <v>91</v>
       </c>
       <c r="E34">
-        <v>4843</v>
+        <v>91</v>
       </c>
       <c r="F34">
         <v>0</v>
       </c>
       <c r="G34">
-        <v>18.2</v>
+        <v>1268</v>
       </c>
       <c r="H34">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I34">
-        <v>33</v>
+        <v>2282</v>
       </c>
       <c r="J34">
-        <v>25</v>
+        <v>1775</v>
       </c>
       <c r="K34">
-        <v>3538</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35">
@@ -1885,28 +1885,28 @@
         <v>100</v>
       </c>
       <c r="D35">
-        <v>4628</v>
+        <v>87</v>
       </c>
       <c r="E35">
-        <v>4628</v>
+        <v>87</v>
       </c>
       <c r="F35">
         <v>0</v>
       </c>
       <c r="G35">
-        <v>18.6</v>
+        <v>1290</v>
       </c>
       <c r="H35">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I35">
-        <v>33</v>
+        <v>2322</v>
       </c>
       <c r="J35">
-        <v>26</v>
+        <v>1806</v>
       </c>
       <c r="K35">
-        <v>3381</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36">
@@ -1920,28 +1920,28 @@
         <v>100</v>
       </c>
       <c r="D36">
-        <v>5362</v>
+        <v>101</v>
       </c>
       <c r="E36">
-        <v>5362</v>
+        <v>101</v>
       </c>
       <c r="F36">
         <v>0</v>
       </c>
       <c r="G36">
-        <v>17.5</v>
+        <v>1214.9</v>
       </c>
       <c r="H36">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I36">
-        <v>32</v>
+        <v>2187</v>
       </c>
       <c r="J36">
-        <v>25</v>
+        <v>1701</v>
       </c>
       <c r="K36">
-        <v>3917</v>
+        <v>82</v>
       </c>
     </row>
     <row r="37">
@@ -1955,28 +1955,28 @@
         <v>100</v>
       </c>
       <c r="D37">
-        <v>4809</v>
+        <v>91</v>
       </c>
       <c r="E37">
-        <v>4809</v>
+        <v>91</v>
       </c>
       <c r="F37">
         <v>0</v>
       </c>
       <c r="G37">
-        <v>18.3</v>
+        <v>1271.5</v>
       </c>
       <c r="H37">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I37">
-        <v>33</v>
+        <v>2289</v>
       </c>
       <c r="J37">
-        <v>26</v>
+        <v>1780</v>
       </c>
       <c r="K37">
-        <v>3513</v>
+        <v>74</v>
       </c>
     </row>
     <row r="38">
@@ -1990,28 +1990,28 @@
         <v>100</v>
       </c>
       <c r="D38">
-        <v>5161</v>
+        <v>97</v>
       </c>
       <c r="E38">
-        <v>5161</v>
+        <v>97</v>
       </c>
       <c r="F38">
         <v>0</v>
       </c>
       <c r="G38">
-        <v>17.8</v>
+        <v>1235.4</v>
       </c>
       <c r="H38">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I38">
-        <v>32</v>
+        <v>2224</v>
       </c>
       <c r="J38">
-        <v>25</v>
+        <v>1730</v>
       </c>
       <c r="K38">
-        <v>3770</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39">
@@ -2025,28 +2025,28 @@
         <v>100</v>
       </c>
       <c r="D39">
-        <v>5585</v>
+        <v>105</v>
       </c>
       <c r="E39">
-        <v>5585</v>
+        <v>105</v>
       </c>
       <c r="F39">
         <v>0</v>
       </c>
       <c r="G39">
-        <v>17.2</v>
+        <v>1192</v>
       </c>
       <c r="H39">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I39">
-        <v>31</v>
+        <v>2146</v>
       </c>
       <c r="J39">
-        <v>24</v>
+        <v>1669</v>
       </c>
       <c r="K39">
-        <v>4080</v>
+        <v>85</v>
       </c>
     </row>
     <row r="40">
@@ -2060,28 +2060,28 @@
         <v>100</v>
       </c>
       <c r="D40">
-        <v>5978</v>
+        <v>113</v>
       </c>
       <c r="E40">
-        <v>5978</v>
+        <v>113</v>
       </c>
       <c r="F40">
         <v>0</v>
       </c>
       <c r="G40">
-        <v>16.6</v>
+        <v>1151.8</v>
       </c>
       <c r="H40">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I40">
-        <v>30</v>
+        <v>2073</v>
       </c>
       <c r="J40">
-        <v>23</v>
+        <v>1613</v>
       </c>
       <c r="K40">
-        <v>4367</v>
+        <v>92</v>
       </c>
     </row>
     <row r="41">
@@ -2095,28 +2095,28 @@
         <v>100</v>
       </c>
       <c r="D41">
-        <v>6989</v>
+        <v>132</v>
       </c>
       <c r="E41">
-        <v>6989</v>
+        <v>132</v>
       </c>
       <c r="F41">
         <v>0</v>
       </c>
       <c r="G41">
-        <v>15.1</v>
+        <v>1048.3</v>
       </c>
       <c r="H41">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I41">
-        <v>27</v>
+        <v>1887</v>
       </c>
       <c r="J41">
-        <v>21</v>
+        <v>1468</v>
       </c>
       <c r="K41">
-        <v>5105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="42">
@@ -2130,28 +2130,28 @@
         <v>100</v>
       </c>
       <c r="D42">
-        <v>6315</v>
+        <v>119</v>
       </c>
       <c r="E42">
-        <v>6315</v>
+        <v>119</v>
       </c>
       <c r="F42">
         <v>0</v>
       </c>
       <c r="G42">
-        <v>16.1</v>
+        <v>1117.3</v>
       </c>
       <c r="H42">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I42">
-        <v>29</v>
+        <v>2011</v>
       </c>
       <c r="J42">
-        <v>23</v>
+        <v>1564</v>
       </c>
       <c r="K42">
-        <v>4613</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43">
@@ -2165,28 +2165,28 @@
         <v>100</v>
       </c>
       <c r="D43">
-        <v>6177</v>
+        <v>117</v>
       </c>
       <c r="E43">
-        <v>6177</v>
+        <v>117</v>
       </c>
       <c r="F43">
         <v>0</v>
       </c>
       <c r="G43">
-        <v>16.3</v>
+        <v>1131.5</v>
       </c>
       <c r="H43">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I43">
-        <v>29</v>
+        <v>2037</v>
       </c>
       <c r="J43">
-        <v>23</v>
+        <v>1584</v>
       </c>
       <c r="K43">
-        <v>4512</v>
+        <v>95</v>
       </c>
     </row>
     <row r="44">
@@ -2200,28 +2200,28 @@
         <v>100</v>
       </c>
       <c r="D44">
-        <v>5863</v>
+        <v>111</v>
       </c>
       <c r="E44">
-        <v>5863</v>
+        <v>111</v>
       </c>
       <c r="F44">
         <v>0</v>
       </c>
       <c r="G44">
-        <v>16.7</v>
+        <v>1163.7</v>
       </c>
       <c r="H44">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I44">
-        <v>30</v>
+        <v>2095</v>
       </c>
       <c r="J44">
-        <v>23</v>
+        <v>1629</v>
       </c>
       <c r="K44">
-        <v>4283</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45">
@@ -2235,28 +2235,28 @@
         <v>100</v>
       </c>
       <c r="D45">
-        <v>5449</v>
+        <v>103</v>
       </c>
       <c r="E45">
-        <v>5449</v>
+        <v>103</v>
       </c>
       <c r="F45">
         <v>0</v>
       </c>
       <c r="G45">
-        <v>17.4</v>
+        <v>1206</v>
       </c>
       <c r="H45">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I45">
-        <v>31</v>
+        <v>2171</v>
       </c>
       <c r="J45">
-        <v>24</v>
+        <v>1688</v>
       </c>
       <c r="K45">
-        <v>3980</v>
+        <v>84</v>
       </c>
     </row>
     <row r="46">
@@ -2270,28 +2270,28 @@
         <v>100</v>
       </c>
       <c r="D46">
-        <v>5783</v>
+        <v>109</v>
       </c>
       <c r="E46">
-        <v>5783</v>
+        <v>109</v>
       </c>
       <c r="F46">
         <v>0</v>
       </c>
       <c r="G46">
-        <v>16.9</v>
+        <v>1171.8</v>
       </c>
       <c r="H46">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I46">
-        <v>30</v>
+        <v>2109</v>
       </c>
       <c r="J46">
-        <v>24</v>
+        <v>1641</v>
       </c>
       <c r="K46">
-        <v>4224</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47">
@@ -2305,28 +2305,28 @@
         <v>100</v>
       </c>
       <c r="D47">
-        <v>4727</v>
+        <v>89</v>
       </c>
       <c r="E47">
-        <v>4727</v>
+        <v>89</v>
       </c>
       <c r="F47">
         <v>0</v>
       </c>
       <c r="G47">
-        <v>18.4</v>
+        <v>1279.9</v>
       </c>
       <c r="H47">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I47">
-        <v>33</v>
+        <v>2304</v>
       </c>
       <c r="J47">
-        <v>26</v>
+        <v>1792</v>
       </c>
       <c r="K47">
-        <v>3453</v>
+        <v>72</v>
       </c>
     </row>
     <row r="48">
@@ -2340,28 +2340,28 @@
         <v>100</v>
       </c>
       <c r="D48">
-        <v>4596</v>
+        <v>87</v>
       </c>
       <c r="E48">
-        <v>4596</v>
+        <v>87</v>
       </c>
       <c r="F48">
         <v>0</v>
       </c>
       <c r="G48">
-        <v>18.6</v>
+        <v>1293.3</v>
       </c>
       <c r="H48">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I48">
-        <v>33</v>
+        <v>2328</v>
       </c>
       <c r="J48">
-        <v>26</v>
+        <v>1811</v>
       </c>
       <c r="K48">
-        <v>3357</v>
+        <v>71</v>
       </c>
     </row>
     <row r="49">
@@ -2375,28 +2375,28 @@
         <v>100</v>
       </c>
       <c r="D49">
-        <v>4676</v>
+        <v>88</v>
       </c>
       <c r="E49">
-        <v>4676</v>
+        <v>88</v>
       </c>
       <c r="F49">
         <v>0</v>
       </c>
       <c r="G49">
-        <v>18.5</v>
+        <v>1285.1</v>
       </c>
       <c r="H49">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I49">
-        <v>33</v>
+        <v>2313</v>
       </c>
       <c r="J49">
-        <v>26</v>
+        <v>1799</v>
       </c>
       <c r="K49">
-        <v>3416</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50">
@@ -2410,28 +2410,28 @@
         <v>100</v>
       </c>
       <c r="D50">
-        <v>4947</v>
+        <v>93</v>
       </c>
       <c r="E50">
-        <v>4947</v>
+        <v>93</v>
       </c>
       <c r="F50">
         <v>0</v>
       </c>
       <c r="G50">
-        <v>18.1</v>
+        <v>1257.4</v>
       </c>
       <c r="H50">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I50">
-        <v>33</v>
+        <v>2263</v>
       </c>
       <c r="J50">
-        <v>25</v>
+        <v>1760</v>
       </c>
       <c r="K50">
-        <v>3614</v>
+        <v>76</v>
       </c>
     </row>
     <row r="51">
@@ -2445,28 +2445,28 @@
         <v>100</v>
       </c>
       <c r="D51">
-        <v>6089</v>
+        <v>115</v>
       </c>
       <c r="E51">
-        <v>6089</v>
+        <v>115</v>
       </c>
       <c r="F51">
         <v>0</v>
       </c>
       <c r="G51">
-        <v>16.4</v>
+        <v>1140.5</v>
       </c>
       <c r="H51">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I51">
-        <v>30</v>
+        <v>2053</v>
       </c>
       <c r="J51">
-        <v>23</v>
+        <v>1597</v>
       </c>
       <c r="K51">
-        <v>4448</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52">
@@ -2480,28 +2480,28 @@
         <v>100</v>
       </c>
       <c r="D52">
-        <v>5766</v>
+        <v>109</v>
       </c>
       <c r="E52">
-        <v>5766</v>
+        <v>109</v>
       </c>
       <c r="F52">
         <v>0</v>
       </c>
       <c r="G52">
-        <v>16.9</v>
+        <v>1173.6</v>
       </c>
       <c r="H52">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I52">
-        <v>30</v>
+        <v>2112</v>
       </c>
       <c r="J52">
-        <v>24</v>
+        <v>1643</v>
       </c>
       <c r="K52">
-        <v>4212</v>
+        <v>89</v>
       </c>
     </row>
     <row r="53">
@@ -2515,28 +2515,28 @@
         <v>100</v>
       </c>
       <c r="D53">
-        <v>6113</v>
+        <v>115</v>
       </c>
       <c r="E53">
-        <v>6113</v>
+        <v>115</v>
       </c>
       <c r="F53">
         <v>0</v>
       </c>
       <c r="G53">
-        <v>16.4</v>
+        <v>1138</v>
       </c>
       <c r="H53">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I53">
-        <v>30</v>
+        <v>2048</v>
       </c>
       <c r="J53">
-        <v>23</v>
+        <v>1593</v>
       </c>
       <c r="K53">
-        <v>4465</v>
+        <v>94</v>
       </c>
     </row>
     <row r="54">
@@ -2550,28 +2550,28 @@
         <v>100</v>
       </c>
       <c r="D54">
-        <v>6300</v>
+        <v>119</v>
       </c>
       <c r="E54">
-        <v>6300</v>
+        <v>119</v>
       </c>
       <c r="F54">
         <v>0</v>
       </c>
       <c r="G54">
-        <v>16.1</v>
+        <v>1118.9</v>
       </c>
       <c r="H54">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I54">
-        <v>29</v>
+        <v>2014</v>
       </c>
       <c r="J54">
-        <v>23</v>
+        <v>1566</v>
       </c>
       <c r="K54">
-        <v>4602</v>
+        <v>97</v>
       </c>
     </row>
     <row r="55">
@@ -2585,28 +2585,28 @@
         <v>100</v>
       </c>
       <c r="D55">
-        <v>6280</v>
+        <v>119</v>
       </c>
       <c r="E55">
-        <v>6280</v>
+        <v>119</v>
       </c>
       <c r="F55">
         <v>0</v>
       </c>
       <c r="G55">
-        <v>16.1</v>
+        <v>1120.9</v>
       </c>
       <c r="H55">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I55">
-        <v>29</v>
+        <v>2018</v>
       </c>
       <c r="J55">
-        <v>23</v>
+        <v>1569</v>
       </c>
       <c r="K55">
-        <v>4587</v>
+        <v>97</v>
       </c>
     </row>
     <row r="56">
@@ -2620,28 +2620,28 @@
         <v>100</v>
       </c>
       <c r="D56">
-        <v>6805</v>
+        <v>128</v>
       </c>
       <c r="E56">
-        <v>6805</v>
+        <v>128</v>
       </c>
       <c r="F56">
         <v>0</v>
       </c>
       <c r="G56">
-        <v>15.4</v>
+        <v>1067.2</v>
       </c>
       <c r="H56">
-        <v>6</v>
+        <v>637</v>
       </c>
       <c r="I56">
-        <v>28</v>
+        <v>1921</v>
       </c>
       <c r="J56">
-        <v>22</v>
+        <v>1494</v>
       </c>
       <c r="K56">
-        <v>4971</v>
+        <v>104</v>
       </c>
     </row>
     <row r="57">
@@ -2655,28 +2655,28 @@
         <v>100</v>
       </c>
       <c r="D57">
-        <v>5690</v>
+        <v>107</v>
       </c>
       <c r="E57">
-        <v>5690</v>
+        <v>107</v>
       </c>
       <c r="F57">
         <v>0</v>
       </c>
       <c r="G57">
-        <v>17</v>
+        <v>1181.4</v>
       </c>
       <c r="H57">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I57">
-        <v>31</v>
+        <v>2127</v>
       </c>
       <c r="J57">
-        <v>24</v>
+        <v>1654</v>
       </c>
       <c r="K57">
-        <v>4156</v>
+        <v>87</v>
       </c>
     </row>
     <row r="58">
@@ -2690,28 +2690,28 @@
         <v>100</v>
       </c>
       <c r="D58">
-        <v>5263</v>
+        <v>99</v>
       </c>
       <c r="E58">
-        <v>5263</v>
+        <v>99</v>
       </c>
       <c r="F58">
         <v>0</v>
       </c>
       <c r="G58">
-        <v>17.6</v>
+        <v>1225</v>
       </c>
       <c r="H58">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I58">
-        <v>32</v>
+        <v>2205</v>
       </c>
       <c r="J58">
-        <v>25</v>
+        <v>1715</v>
       </c>
       <c r="K58">
-        <v>3845</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59">
@@ -2725,28 +2725,28 @@
         <v>100</v>
       </c>
       <c r="D59">
-        <v>4885</v>
+        <v>92</v>
       </c>
       <c r="E59">
-        <v>4885</v>
+        <v>92</v>
       </c>
       <c r="F59">
         <v>0</v>
       </c>
       <c r="G59">
-        <v>18.2</v>
+        <v>1263.8</v>
       </c>
       <c r="H59">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I59">
-        <v>33</v>
+        <v>2275</v>
       </c>
       <c r="J59">
-        <v>25</v>
+        <v>1769</v>
       </c>
       <c r="K59">
-        <v>3568</v>
+        <v>75</v>
       </c>
     </row>
     <row r="60">
@@ -2760,28 +2760,28 @@
         <v>100</v>
       </c>
       <c r="D60">
-        <v>4646</v>
+        <v>88</v>
       </c>
       <c r="E60">
-        <v>4646</v>
+        <v>88</v>
       </c>
       <c r="F60">
         <v>0</v>
       </c>
       <c r="G60">
-        <v>18.5</v>
+        <v>1288.2</v>
       </c>
       <c r="H60">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I60">
-        <v>33</v>
+        <v>2319</v>
       </c>
       <c r="J60">
-        <v>26</v>
+        <v>1803</v>
       </c>
       <c r="K60">
-        <v>3394</v>
+        <v>72</v>
       </c>
     </row>
     <row r="61">
@@ -2795,28 +2795,28 @@
         <v>100</v>
       </c>
       <c r="D61">
-        <v>5352</v>
+        <v>101</v>
       </c>
       <c r="E61">
-        <v>5352</v>
+        <v>101</v>
       </c>
       <c r="F61">
         <v>0</v>
       </c>
       <c r="G61">
-        <v>17.5</v>
+        <v>1215.9</v>
       </c>
       <c r="H61">
-        <v>7</v>
+        <v>637</v>
       </c>
       <c r="I61">
-        <v>32</v>
+        <v>2189</v>
       </c>
       <c r="J61">
-        <v>25</v>
+        <v>1702</v>
       </c>
       <c r="K61">
-        <v>3910</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2847,7 +2847,7 @@
         <v>1.00% (Fastest 1%)</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>637</v>
       </c>
     </row>
     <row r="3">
@@ -2855,7 +2855,7 @@
         <v>5.00%</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>764</v>
       </c>
     </row>
     <row r="4">
@@ -2863,7 +2863,7 @@
         <v>10.00%</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>956</v>
       </c>
     </row>
     <row r="5">
@@ -2871,7 +2871,7 @@
         <v>25.00% (Q1)</v>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>823</v>
       </c>
     </row>
     <row r="6">
@@ -2879,7 +2879,7 @@
         <v>50.00% (Median / P50)</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="7">
@@ -2887,7 +2887,7 @@
         <v>75.00% (Q3)</v>
       </c>
       <c r="B7">
-        <v>20</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="8">
@@ -2895,7 +2895,7 @@
         <v>90.00% (P90)</v>
       </c>
       <c r="B8">
-        <v>24</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="9">
@@ -2903,7 +2903,7 @@
         <v>95.00% (P95)</v>
       </c>
       <c r="B9">
-        <v>35</v>
+        <v>3498</v>
       </c>
     </row>
     <row r="10">
@@ -2911,7 +2911,7 @@
         <v>97.50%</v>
       </c>
       <c r="B10">
-        <v>39</v>
+        <v>3551</v>
       </c>
     </row>
     <row r="11">
@@ -2919,7 +2919,7 @@
         <v>99.00% (P99)</v>
       </c>
       <c r="B11">
-        <v>43</v>
+        <v>3604</v>
       </c>
     </row>
     <row r="12">
@@ -2927,7 +2927,7 @@
         <v>99.90% (P99.9)</v>
       </c>
       <c r="B12">
-        <v>54</v>
+        <v>4505</v>
       </c>
     </row>
     <row r="13">
@@ -2935,7 +2935,7 @@
         <v>100.00% (Max / Slowest)</v>
       </c>
       <c r="B13">
-        <v>1471</v>
+        <v>5057</v>
       </c>
     </row>
   </sheetData>
@@ -2977,10 +2977,10 @@
         <v>Success</v>
       </c>
       <c r="C2">
-        <v>99</v>
+        <v>5096</v>
       </c>
       <c r="D2" t="str">
-        <v>0.03%</v>
+        <v>100.00%</v>
       </c>
     </row>
     <row r="3">
@@ -2991,7 +2991,7 @@
         <v>Client Error</v>
       </c>
       <c r="C3">
-        <v>344481</v>
+        <v>0</v>
       </c>
       <c r="D3" t="str">
         <v>0.00%</v>

</xml_diff>